<commit_message>
Pocetak elektronskog zavrsnog racuna
</commit_message>
<xml_diff>
--- a/stanje_konta.xlsx
+++ b/stanje_konta.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Oznaka</t>
   </si>
@@ -28,136 +28,79 @@
     <t>Saldo</t>
   </si>
   <si>
-    <t>121113</t>
-  </si>
-  <si>
-    <t>123221</t>
-  </si>
-  <si>
-    <t>123231</t>
-  </si>
-  <si>
-    <t>131211</t>
-  </si>
-  <si>
-    <t>231111</t>
-  </si>
-  <si>
-    <t>231211</t>
-  </si>
-  <si>
-    <t>231311</t>
-  </si>
-  <si>
-    <t>231411</t>
-  </si>
-  <si>
-    <t>231511</t>
-  </si>
-  <si>
-    <t>234111</t>
-  </si>
-  <si>
-    <t>234211</t>
-  </si>
-  <si>
-    <t>252111</t>
-  </si>
-  <si>
-    <t>291211</t>
-  </si>
-  <si>
-    <t>291213</t>
-  </si>
-  <si>
-    <t>411111</t>
-  </si>
-  <si>
-    <t>411115</t>
-  </si>
-  <si>
-    <t>411117</t>
-  </si>
-  <si>
-    <t>411118</t>
-  </si>
-  <si>
-    <t>412111</t>
-  </si>
-  <si>
-    <t>412211</t>
-  </si>
-  <si>
-    <t>421211</t>
-  </si>
-  <si>
-    <t>421225</t>
-  </si>
-  <si>
-    <t>421311</t>
-  </si>
-  <si>
-    <t>421322</t>
-  </si>
-  <si>
-    <t>421323</t>
-  </si>
-  <si>
-    <t>421324</t>
-  </si>
-  <si>
-    <t>421325</t>
-  </si>
-  <si>
-    <t>421411</t>
-  </si>
-  <si>
-    <t>421412</t>
-  </si>
-  <si>
-    <t>421414</t>
-  </si>
-  <si>
-    <t>421511</t>
-  </si>
-  <si>
-    <t>421621</t>
-  </si>
-  <si>
-    <t>421911</t>
-  </si>
-  <si>
-    <t>423711</t>
-  </si>
-  <si>
-    <t>423911</t>
-  </si>
-  <si>
-    <t>425117</t>
-  </si>
-  <si>
-    <t>425119</t>
-  </si>
-  <si>
-    <t>425229</t>
-  </si>
-  <si>
-    <t>426111</t>
-  </si>
-  <si>
-    <t>426311</t>
-  </si>
-  <si>
-    <t>426412</t>
-  </si>
-  <si>
-    <t>426819</t>
-  </si>
-  <si>
-    <t>426919</t>
-  </si>
-  <si>
-    <t>791111</t>
+    <t>0112</t>
+  </si>
+  <si>
+    <t>0161</t>
+  </si>
+  <si>
+    <t>1232</t>
+  </si>
+  <si>
+    <t>1312</t>
+  </si>
+  <si>
+    <t>2311</t>
+  </si>
+  <si>
+    <t>2312</t>
+  </si>
+  <si>
+    <t>2313</t>
+  </si>
+  <si>
+    <t>2314</t>
+  </si>
+  <si>
+    <t>2315</t>
+  </si>
+  <si>
+    <t>2321</t>
+  </si>
+  <si>
+    <t>2322</t>
+  </si>
+  <si>
+    <t>2331</t>
+  </si>
+  <si>
+    <t>2332</t>
+  </si>
+  <si>
+    <t>2341</t>
+  </si>
+  <si>
+    <t>2342</t>
+  </si>
+  <si>
+    <t>2361</t>
+  </si>
+  <si>
+    <t>2362</t>
+  </si>
+  <si>
+    <t>2363</t>
+  </si>
+  <si>
+    <t>2364</t>
+  </si>
+  <si>
+    <t>2365</t>
+  </si>
+  <si>
+    <t>2521</t>
+  </si>
+  <si>
+    <t>2912</t>
+  </si>
+  <si>
+    <t>3111</t>
+  </si>
+  <si>
+    <t>3511</t>
+  </si>
+  <si>
+    <t>3521</t>
   </si>
 </sst>
 </file>
@@ -515,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -537,13 +480,13 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>3676095.92</v>
+        <v>8053976.1</v>
       </c>
       <c r="C2">
-        <v>3676095.92</v>
+        <v>6628787.02</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1425189.08</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -551,13 +494,13 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>76048.8</v>
+        <v>320907.5</v>
       </c>
       <c r="C3">
-        <v>44609.17</v>
+        <v>0</v>
       </c>
       <c r="D3">
-        <v>31439.63</v>
+        <v>320907.5</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -565,13 +508,13 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>1686447.18</v>
       </c>
       <c r="C4">
-        <v>126744</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>-126744</v>
+        <v>1686447.18</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -579,13 +522,13 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>3571481.76</v>
+        <v>2938690.84</v>
       </c>
       <c r="C5">
-        <v>3676095.92</v>
+        <v>0</v>
       </c>
       <c r="D5">
-        <v>-104614.16</v>
+        <v>2938690.84</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -593,13 +536,13 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>1613666.39</v>
+        <v>0</v>
       </c>
       <c r="C6">
-        <v>1613666.39</v>
+        <v>1139932.37</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>-1139932.37</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -607,13 +550,13 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>169591.35</v>
+        <v>0</v>
       </c>
       <c r="C7">
-        <v>169591.35</v>
+        <v>121379.02</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>-121379.02</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -621,13 +564,13 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>311537.4</v>
+        <v>0</v>
       </c>
       <c r="C8">
-        <v>311537.4</v>
+        <v>220327.73</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>-220327.73</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -635,13 +578,13 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>114601.26</v>
+        <v>0</v>
       </c>
       <c r="C9">
-        <v>114601.26</v>
+        <v>81049.14</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>-81049.14</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -649,13 +592,13 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>15870.52</v>
+        <v>0</v>
       </c>
       <c r="C10">
-        <v>15870.52</v>
+        <v>11081.26</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>-11081.26</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -663,13 +606,13 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>222526.7</v>
+        <v>0</v>
       </c>
       <c r="C11">
-        <v>222526.7</v>
+        <v>57489.04</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>-57489.04</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -677,13 +620,13 @@
         <v>14</v>
       </c>
       <c r="B12">
-        <v>114601.26</v>
+        <v>0</v>
       </c>
       <c r="C12">
-        <v>114601.26</v>
+        <v>2307.45</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>-2307.45</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -691,13 +634,13 @@
         <v>15</v>
       </c>
       <c r="B13">
-        <v>1113701.04</v>
+        <v>0</v>
       </c>
       <c r="C13">
-        <v>1009086.88</v>
+        <v>286499.79</v>
       </c>
       <c r="D13">
-        <v>104614.16</v>
+        <v>-286499.79</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -705,13 +648,13 @@
         <v>16</v>
       </c>
       <c r="B14">
-        <v>44609.17</v>
+        <v>0</v>
       </c>
       <c r="C14">
-        <v>76048.8</v>
+        <v>28705.31</v>
       </c>
       <c r="D14">
-        <v>-31439.63</v>
+        <v>-28705.31</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -719,13 +662,13 @@
         <v>17</v>
       </c>
       <c r="B15">
-        <v>126744</v>
+        <v>0</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>157376.97</v>
       </c>
       <c r="D15">
-        <v>126744</v>
+        <v>-157376.97</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -733,13 +676,13 @@
         <v>18</v>
       </c>
       <c r="B16">
-        <v>1695100.35</v>
+        <v>0</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>81049.14</v>
       </c>
       <c r="D16">
-        <v>1695100.35</v>
+        <v>-81049.14</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -747,13 +690,13 @@
         <v>19</v>
       </c>
       <c r="B17">
-        <v>158315.51</v>
+        <v>0</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>43360</v>
       </c>
       <c r="D17">
-        <v>158315.51</v>
+        <v>-43360</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -761,13 +704,13 @@
         <v>20</v>
       </c>
       <c r="B18">
-        <v>15463.6</v>
+        <v>0</v>
       </c>
       <c r="C18">
-        <v>0</v>
+        <v>3232.94</v>
       </c>
       <c r="D18">
-        <v>15463.6</v>
+        <v>-3232.94</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -775,13 +718,13 @@
         <v>21</v>
       </c>
       <c r="B19">
-        <v>356387.46</v>
+        <v>0</v>
       </c>
       <c r="C19">
-        <v>0</v>
+        <v>13960.43</v>
       </c>
       <c r="D19">
-        <v>356387.46</v>
+        <v>-13960.43</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -789,13 +732,13 @@
         <v>22</v>
       </c>
       <c r="B20">
-        <v>222526.7</v>
+        <v>0</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>5991.36</v>
       </c>
       <c r="D20">
-        <v>222526.7</v>
+        <v>-5991.36</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -803,13 +746,13 @@
         <v>23</v>
       </c>
       <c r="B21">
-        <v>114601.26</v>
+        <v>0</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>436.26</v>
       </c>
       <c r="D21">
-        <v>114601.26</v>
+        <v>-436.26</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -817,13 +760,13 @@
         <v>24</v>
       </c>
       <c r="B22">
-        <v>3262.34</v>
+        <v>0</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>684512.63</v>
       </c>
       <c r="D22">
-        <v>3262.34</v>
+        <v>-684512.63</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -831,13 +774,13 @@
         <v>25</v>
       </c>
       <c r="B23">
-        <v>50351.2</v>
+        <v>0</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>1686447.18</v>
       </c>
       <c r="D23">
-        <v>50351.2</v>
+        <v>-1686447.18</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -845,13 +788,13 @@
         <v>26</v>
       </c>
       <c r="B24">
-        <v>15269.85</v>
+        <v>0</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>1746096.58</v>
       </c>
       <c r="D24">
-        <v>15269.85</v>
+        <v>-1746096.58</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -859,13 +802,13 @@
         <v>27</v>
       </c>
       <c r="B25">
-        <v>3732</v>
+        <v>244538.88</v>
       </c>
       <c r="C25">
         <v>0</v>
       </c>
       <c r="D25">
-        <v>3732</v>
+        <v>244538.88</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -873,279 +816,13 @@
         <v>28</v>
       </c>
       <c r="B26">
-        <v>196554.72</v>
+        <v>0</v>
       </c>
       <c r="C26">
-        <v>0</v>
+        <v>244538.88</v>
       </c>
       <c r="D26">
-        <v>196554.72</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="A27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B27">
-        <v>44664.58</v>
-      </c>
-      <c r="C27">
-        <v>0</v>
-      </c>
-      <c r="D27">
-        <v>44664.58</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28">
-        <v>199996.8</v>
-      </c>
-      <c r="C28">
-        <v>0</v>
-      </c>
-      <c r="D28">
-        <v>199996.8</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4">
-      <c r="A29" t="s">
-        <v>31</v>
-      </c>
-      <c r="B29">
-        <v>32605.55</v>
-      </c>
-      <c r="C29">
-        <v>0</v>
-      </c>
-      <c r="D29">
-        <v>32605.55</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="A30" t="s">
-        <v>32</v>
-      </c>
-      <c r="B30">
-        <v>11796</v>
-      </c>
-      <c r="C30">
-        <v>0</v>
-      </c>
-      <c r="D30">
-        <v>11796</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" t="s">
-        <v>33</v>
-      </c>
-      <c r="B31">
-        <v>32744.96</v>
-      </c>
-      <c r="C31">
-        <v>0</v>
-      </c>
-      <c r="D31">
-        <v>32744.96</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="A32" t="s">
-        <v>34</v>
-      </c>
-      <c r="B32">
-        <v>4622.8</v>
-      </c>
-      <c r="C32">
-        <v>0</v>
-      </c>
-      <c r="D32">
-        <v>4622.8</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4">
-      <c r="A33" t="s">
-        <v>35</v>
-      </c>
-      <c r="B33">
-        <v>185640</v>
-      </c>
-      <c r="C33">
-        <v>0</v>
-      </c>
-      <c r="D33">
-        <v>185640</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="A34" t="s">
-        <v>36</v>
-      </c>
-      <c r="B34">
-        <v>1131.6</v>
-      </c>
-      <c r="C34">
-        <v>0</v>
-      </c>
-      <c r="D34">
-        <v>1131.6</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4">
-      <c r="A35" t="s">
-        <v>37</v>
-      </c>
-      <c r="B35">
-        <v>28742.2</v>
-      </c>
-      <c r="C35">
-        <v>0</v>
-      </c>
-      <c r="D35">
-        <v>28742.2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4">
-      <c r="A36" t="s">
-        <v>38</v>
-      </c>
-      <c r="B36">
-        <v>3806</v>
-      </c>
-      <c r="C36">
-        <v>0</v>
-      </c>
-      <c r="D36">
-        <v>3806</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4">
-      <c r="A37" t="s">
-        <v>39</v>
-      </c>
-      <c r="B37">
-        <v>1945.44</v>
-      </c>
-      <c r="C37">
-        <v>0</v>
-      </c>
-      <c r="D37">
-        <v>1945.44</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="A38" t="s">
-        <v>40</v>
-      </c>
-      <c r="B38">
-        <v>2983</v>
-      </c>
-      <c r="C38">
-        <v>0</v>
-      </c>
-      <c r="D38">
-        <v>2983</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="A39" t="s">
-        <v>41</v>
-      </c>
-      <c r="B39">
-        <v>1500</v>
-      </c>
-      <c r="C39">
-        <v>0</v>
-      </c>
-      <c r="D39">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="A40" t="s">
-        <v>42</v>
-      </c>
-      <c r="B40">
-        <v>100656</v>
-      </c>
-      <c r="C40">
-        <v>0</v>
-      </c>
-      <c r="D40">
-        <v>100656</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4">
-      <c r="A41" t="s">
-        <v>43</v>
-      </c>
-      <c r="B41">
-        <v>47300</v>
-      </c>
-      <c r="C41">
-        <v>0</v>
-      </c>
-      <c r="D41">
-        <v>47300</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4">
-      <c r="A42" t="s">
-        <v>44</v>
-      </c>
-      <c r="B42">
-        <v>76048.8</v>
-      </c>
-      <c r="C42">
-        <v>0</v>
-      </c>
-      <c r="D42">
-        <v>76048.8</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4">
-      <c r="A43" t="s">
-        <v>45</v>
-      </c>
-      <c r="B43">
-        <v>41947.2</v>
-      </c>
-      <c r="C43">
-        <v>0</v>
-      </c>
-      <c r="D43">
-        <v>41947.2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4">
-      <c r="A44" t="s">
-        <v>46</v>
-      </c>
-      <c r="B44">
-        <v>26400</v>
-      </c>
-      <c r="C44">
-        <v>0</v>
-      </c>
-      <c r="D44">
-        <v>26400</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4">
-      <c r="A45" t="s">
-        <v>47</v>
-      </c>
-      <c r="B45">
-        <v>0</v>
-      </c>
-      <c r="C45">
-        <v>3676095.92</v>
-      </c>
-      <c r="D45">
-        <v>-3676095.92</v>
+        <v>-244538.88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
pravljenje elektrnskog zavrsnog racuna
</commit_message>
<xml_diff>
--- a/stanje_konta.xlsx
+++ b/stanje_konta.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>Oznaka</t>
   </si>
@@ -34,6 +34,15 @@
     <t>0161</t>
   </si>
   <si>
+    <t>0221</t>
+  </si>
+  <si>
+    <t>1211</t>
+  </si>
+  <si>
+    <t>1221</t>
+  </si>
+  <si>
     <t>1232</t>
   </si>
   <si>
@@ -73,6 +82,9 @@
     <t>2342</t>
   </si>
   <si>
+    <t>2351</t>
+  </si>
+  <si>
     <t>2361</t>
   </si>
   <si>
@@ -94,13 +106,112 @@
     <t>2912</t>
   </si>
   <si>
+    <t>2919</t>
+  </si>
+  <si>
     <t>3111</t>
   </si>
   <si>
+    <t>3112</t>
+  </si>
+  <si>
+    <t>3211</t>
+  </si>
+  <si>
     <t>3511</t>
   </si>
   <si>
     <t>3521</t>
+  </si>
+  <si>
+    <t>4111</t>
+  </si>
+  <si>
+    <t>4121</t>
+  </si>
+  <si>
+    <t>4122</t>
+  </si>
+  <si>
+    <t>4131</t>
+  </si>
+  <si>
+    <t>4143</t>
+  </si>
+  <si>
+    <t>4144</t>
+  </si>
+  <si>
+    <t>4151</t>
+  </si>
+  <si>
+    <t>4161</t>
+  </si>
+  <si>
+    <t>4212</t>
+  </si>
+  <si>
+    <t>4213</t>
+  </si>
+  <si>
+    <t>4214</t>
+  </si>
+  <si>
+    <t>4215</t>
+  </si>
+  <si>
+    <t>4216</t>
+  </si>
+  <si>
+    <t>4219</t>
+  </si>
+  <si>
+    <t>4221</t>
+  </si>
+  <si>
+    <t>4232</t>
+  </si>
+  <si>
+    <t>4233</t>
+  </si>
+  <si>
+    <t>4234</t>
+  </si>
+  <si>
+    <t>4236</t>
+  </si>
+  <si>
+    <t>4237</t>
+  </si>
+  <si>
+    <t>4239</t>
+  </si>
+  <si>
+    <t>4243</t>
+  </si>
+  <si>
+    <t>4251</t>
+  </si>
+  <si>
+    <t>4252</t>
+  </si>
+  <si>
+    <t>4261</t>
+  </si>
+  <si>
+    <t>4263</t>
+  </si>
+  <si>
+    <t>4264</t>
+  </si>
+  <si>
+    <t>4268</t>
+  </si>
+  <si>
+    <t>4269</t>
+  </si>
+  <si>
+    <t>7911</t>
   </si>
 </sst>
 </file>
@@ -458,7 +569,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -480,10 +591,10 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>8053976.1</v>
+        <v>13702459.03</v>
       </c>
       <c r="C2">
-        <v>6628787.02</v>
+        <v>12277269.95</v>
       </c>
       <c r="D2">
         <v>1425189.08</v>
@@ -508,13 +619,13 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>1686447.18</v>
+        <v>53750</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>53750</v>
       </c>
       <c r="D4">
-        <v>1686447.18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -522,13 +633,13 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>2938690.84</v>
+        <v>32483682.56</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>32483682.56</v>
       </c>
       <c r="D5">
-        <v>2938690.84</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -539,10 +650,10 @@
         <v>0</v>
       </c>
       <c r="C6">
-        <v>1139932.37</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <v>-1139932.37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -550,13 +661,13 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>2770346.77</v>
       </c>
       <c r="C7">
-        <v>121379.02</v>
+        <v>1083899.59</v>
       </c>
       <c r="D7">
-        <v>-121379.02</v>
+        <v>1686447.18</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -564,13 +675,13 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>35421393.21</v>
       </c>
       <c r="C8">
-        <v>220327.73</v>
+        <v>32482702.37</v>
       </c>
       <c r="D8">
-        <v>-220327.73</v>
+        <v>2938690.84</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -578,13 +689,13 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>13477956.09</v>
       </c>
       <c r="C9">
-        <v>81049.14</v>
+        <v>14617888.46</v>
       </c>
       <c r="D9">
-        <v>-81049.14</v>
+        <v>-1139932.37</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -592,13 +703,13 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>1436844.84</v>
       </c>
       <c r="C10">
-        <v>11081.26</v>
+        <v>1558223.86</v>
       </c>
       <c r="D10">
-        <v>-11081.26</v>
+        <v>-121379.02</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -606,13 +717,13 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>2605679.29</v>
       </c>
       <c r="C11">
-        <v>57489.04</v>
+        <v>2826007.02</v>
       </c>
       <c r="D11">
-        <v>-57489.04</v>
+        <v>-220327.73</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -620,13 +731,13 @@
         <v>14</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>958517.72</v>
       </c>
       <c r="C12">
-        <v>2307.45</v>
+        <v>1039566.86</v>
       </c>
       <c r="D12">
-        <v>-2307.45</v>
+        <v>-81049.14</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -634,13 +745,13 @@
         <v>15</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>132996.72</v>
       </c>
       <c r="C13">
-        <v>286499.79</v>
+        <v>144077.98</v>
       </c>
       <c r="D13">
-        <v>-286499.79</v>
+        <v>-11081.26</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -648,13 +759,13 @@
         <v>16</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>556429.55</v>
       </c>
       <c r="C14">
-        <v>28705.31</v>
+        <v>613918.59</v>
       </c>
       <c r="D14">
-        <v>-28705.31</v>
+        <v>-57489.04</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -662,13 +773,13 @@
         <v>17</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>19736.71</v>
       </c>
       <c r="C15">
-        <v>157376.97</v>
+        <v>22044.16</v>
       </c>
       <c r="D15">
-        <v>-157376.97</v>
+        <v>-2307.45</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -676,13 +787,13 @@
         <v>18</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>339053</v>
       </c>
       <c r="C16">
-        <v>81049.14</v>
+        <v>625552.79</v>
       </c>
       <c r="D16">
-        <v>-81049.14</v>
+        <v>-286499.79</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -690,13 +801,13 @@
         <v>19</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>31674.56</v>
       </c>
       <c r="C17">
-        <v>43360</v>
+        <v>60379.87</v>
       </c>
       <c r="D17">
-        <v>-43360</v>
+        <v>-28705.31</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -704,13 +815,13 @@
         <v>20</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>1861199.55</v>
       </c>
       <c r="C18">
-        <v>3232.94</v>
+        <v>2018576.52</v>
       </c>
       <c r="D18">
-        <v>-3232.94</v>
+        <v>-157376.97</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -718,13 +829,13 @@
         <v>21</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>958517.72</v>
       </c>
       <c r="C19">
-        <v>13960.43</v>
+        <v>1039566.86</v>
       </c>
       <c r="D19">
-        <v>-13960.43</v>
+        <v>-81049.14</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -732,13 +843,13 @@
         <v>22</v>
       </c>
       <c r="B20">
-        <v>0</v>
+        <v>54000</v>
       </c>
       <c r="C20">
-        <v>5991.36</v>
+        <v>54000</v>
       </c>
       <c r="D20">
-        <v>-5991.36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -746,13 +857,13 @@
         <v>23</v>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>397566</v>
       </c>
       <c r="C21">
-        <v>436.26</v>
+        <v>440926</v>
       </c>
       <c r="D21">
-        <v>-436.26</v>
+        <v>-43360</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -760,13 +871,13 @@
         <v>24</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>8668.219999999999</v>
       </c>
       <c r="C22">
-        <v>684512.63</v>
+        <v>11901.16</v>
       </c>
       <c r="D22">
-        <v>-684512.63</v>
+        <v>-3232.94</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -777,10 +888,10 @@
         <v>0</v>
       </c>
       <c r="C23">
-        <v>1686447.18</v>
+        <v>13960.43</v>
       </c>
       <c r="D23">
-        <v>-1686447.18</v>
+        <v>-13960.43</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -791,10 +902,10 @@
         <v>0</v>
       </c>
       <c r="C24">
-        <v>1746096.58</v>
+        <v>5991.36</v>
       </c>
       <c r="D24">
-        <v>-1746096.58</v>
+        <v>-5991.36</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -802,13 +913,13 @@
         <v>27</v>
       </c>
       <c r="B25">
-        <v>244538.88</v>
+        <v>0</v>
       </c>
       <c r="C25">
-        <v>0</v>
+        <v>436.26</v>
       </c>
       <c r="D25">
-        <v>244538.88</v>
+        <v>-436.26</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -816,13 +927,531 @@
         <v>28</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>9982915.4</v>
       </c>
       <c r="C26">
+        <v>10667428.03</v>
+      </c>
+      <c r="D26">
+        <v>-684512.63</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27">
+        <v>1083899.59</v>
+      </c>
+      <c r="C27">
+        <v>2770346.77</v>
+      </c>
+      <c r="D27">
+        <v>-1686447.18</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29">
+        <v>563135.73</v>
+      </c>
+      <c r="C29">
+        <v>2309232.31</v>
+      </c>
+      <c r="D29">
+        <v>-1746096.58</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30">
+        <v>53750</v>
+      </c>
+      <c r="C30">
+        <v>53750</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31">
+        <v>32482973.87</v>
+      </c>
+      <c r="C31">
+        <v>32482973.87</v>
+      </c>
+      <c r="D31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32">
         <v>244538.88</v>
       </c>
-      <c r="D26">
+      <c r="C32">
+        <v>0</v>
+      </c>
+      <c r="D32">
+        <v>244538.88</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33">
+        <v>0</v>
+      </c>
+      <c r="C33">
+        <v>244538.88</v>
+      </c>
+      <c r="D33">
         <v>-244538.88</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34">
+        <v>18611994.66</v>
+      </c>
+      <c r="C34">
+        <v>18611994.66</v>
+      </c>
+      <c r="D34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35">
+        <v>1861199.55</v>
+      </c>
+      <c r="C35">
+        <v>1861199.55</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36">
+        <v>958517.72</v>
+      </c>
+      <c r="C36">
+        <v>958517.72</v>
+      </c>
+      <c r="D36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37">
+        <v>54000</v>
+      </c>
+      <c r="C37">
+        <v>54000</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38">
+        <v>265566</v>
+      </c>
+      <c r="C38">
+        <v>265566</v>
+      </c>
+      <c r="D38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39">
+        <v>140668.22</v>
+      </c>
+      <c r="C39">
+        <v>140668.22</v>
+      </c>
+      <c r="D39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40">
+        <v>576166.26</v>
+      </c>
+      <c r="C40">
+        <v>576166.26</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41">
+        <v>370727.56</v>
+      </c>
+      <c r="C41">
+        <v>370727.56</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42">
+        <v>740509.5</v>
+      </c>
+      <c r="C42">
+        <v>740509.5</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43">
+        <v>2677291.14</v>
+      </c>
+      <c r="C43">
+        <v>2677291.14</v>
+      </c>
+      <c r="D43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44">
+        <v>1996554.4</v>
+      </c>
+      <c r="C44">
+        <v>1996554.4</v>
+      </c>
+      <c r="D44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45">
+        <v>87348.53999999999</v>
+      </c>
+      <c r="C45">
+        <v>87348.53999999999</v>
+      </c>
+      <c r="D45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46">
+        <v>1447894.27</v>
+      </c>
+      <c r="C46">
+        <v>1447894.27</v>
+      </c>
+      <c r="D46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47">
+        <v>6060.06</v>
+      </c>
+      <c r="C47">
+        <v>6060.06</v>
+      </c>
+      <c r="D47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48">
+        <v>47000</v>
+      </c>
+      <c r="C48">
+        <v>47000</v>
+      </c>
+      <c r="D48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49">
+        <v>400000</v>
+      </c>
+      <c r="C49">
+        <v>400000</v>
+      </c>
+      <c r="D49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50">
+        <v>499200</v>
+      </c>
+      <c r="C50">
+        <v>499200</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51">
+        <v>71366.39999999999</v>
+      </c>
+      <c r="C51">
+        <v>71366.39999999999</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
+      <c r="A52" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52">
+        <v>374000</v>
+      </c>
+      <c r="C52">
+        <v>374000</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53">
+        <v>128190.54</v>
+      </c>
+      <c r="C53">
+        <v>128190.54</v>
+      </c>
+      <c r="D53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
+      <c r="A54" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54">
+        <v>24944</v>
+      </c>
+      <c r="C54">
+        <v>24944</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
+      <c r="A55" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55">
+        <v>200000</v>
+      </c>
+      <c r="C55">
+        <v>200000</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
+      <c r="A56" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56">
+        <v>65077.55</v>
+      </c>
+      <c r="C56">
+        <v>65077.55</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57">
+        <v>1500</v>
+      </c>
+      <c r="C57">
+        <v>1500</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
+      <c r="A58" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58">
+        <v>594786</v>
+      </c>
+      <c r="C58">
+        <v>594786</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="A59" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59">
+        <v>47300</v>
+      </c>
+      <c r="C59">
+        <v>47300</v>
+      </c>
+      <c r="D59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60">
+        <v>113488.8</v>
+      </c>
+      <c r="C60">
+        <v>113488.8</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61">
+        <v>41947.2</v>
+      </c>
+      <c r="C61">
+        <v>41947.2</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62">
+        <v>79404</v>
+      </c>
+      <c r="C62">
+        <v>79404</v>
+      </c>
+      <c r="D62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63">
+        <v>32482702.37</v>
+      </c>
+      <c r="C63">
+        <v>32482702.37</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
izmena elektronskih obrazaca za zavrsni racun
</commit_message>
<xml_diff>
--- a/stanje_konta.xlsx
+++ b/stanje_konta.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
   <si>
     <t>Oznaka</t>
   </si>
@@ -31,6 +31,9 @@
     <t>0112</t>
   </si>
   <si>
+    <t>0151</t>
+  </si>
+  <si>
     <t>0161</t>
   </si>
   <si>
@@ -100,6 +103,9 @@
     <t>2365</t>
   </si>
   <si>
+    <t>2455</t>
+  </si>
+  <si>
     <t>2521</t>
   </si>
   <si>
@@ -115,9 +121,6 @@
     <t>3112</t>
   </si>
   <si>
-    <t>3211</t>
-  </si>
-  <si>
     <t>3511</t>
   </si>
   <si>
@@ -136,12 +139,12 @@
     <t>4131</t>
   </si>
   <si>
+    <t>4141</t>
+  </si>
+  <si>
     <t>4143</t>
   </si>
   <si>
-    <t>4144</t>
-  </si>
-  <si>
     <t>4151</t>
   </si>
   <si>
@@ -172,24 +175,12 @@
     <t>4232</t>
   </si>
   <si>
-    <t>4233</t>
-  </si>
-  <si>
-    <t>4234</t>
-  </si>
-  <si>
-    <t>4236</t>
-  </si>
-  <si>
     <t>4237</t>
   </si>
   <si>
     <t>4239</t>
   </si>
   <si>
-    <t>4243</t>
-  </si>
-  <si>
     <t>4251</t>
   </si>
   <si>
@@ -209,6 +200,12 @@
   </si>
   <si>
     <t>4269</t>
+  </si>
+  <si>
+    <t>4851</t>
+  </si>
+  <si>
+    <t>5122</t>
   </si>
   <si>
     <t>7911</t>
@@ -569,7 +566,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -591,13 +588,13 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>13702459.03</v>
+        <v>8420794.300000001</v>
       </c>
       <c r="C2">
-        <v>12277269.95</v>
+        <v>7203703.51</v>
       </c>
       <c r="D2">
-        <v>1425189.08</v>
+        <v>1217090.79</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -605,13 +602,13 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>320907.5</v>
+        <v>313938.2</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>313938.2</v>
       </c>
       <c r="D3">
-        <v>320907.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -619,13 +616,13 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>53750</v>
+        <v>320907.5</v>
       </c>
       <c r="C4">
-        <v>53750</v>
+        <v>0</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>320907.5</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -633,10 +630,10 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>32483682.56</v>
+        <v>4400</v>
       </c>
       <c r="C5">
-        <v>32483682.56</v>
+        <v>4400</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -647,10 +644,10 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>33678008.31</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>33678008.31</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -661,13 +658,13 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>2770346.77</v>
+        <v>312014.11</v>
       </c>
       <c r="C7">
-        <v>1083899.59</v>
+        <v>312014.11</v>
       </c>
       <c r="D7">
-        <v>1686447.18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -675,13 +672,13 @@
         <v>10</v>
       </c>
       <c r="B8">
-        <v>35421393.21</v>
+        <v>2468034</v>
       </c>
       <c r="C8">
-        <v>32482702.37</v>
+        <v>1601443.78</v>
       </c>
       <c r="D8">
-        <v>2938690.84</v>
+        <v>866590.22</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -689,13 +686,13 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>13477956.09</v>
+        <v>36301165.52</v>
       </c>
       <c r="C9">
-        <v>14617888.46</v>
+        <v>33678008.31</v>
       </c>
       <c r="D9">
-        <v>-1139932.37</v>
+        <v>2623157.21</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -703,13 +700,13 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>1436844.84</v>
+        <v>13876120.16</v>
       </c>
       <c r="C10">
-        <v>1558223.86</v>
+        <v>14986449.92</v>
       </c>
       <c r="D10">
-        <v>-121379.02</v>
+        <v>-1110329.76</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -717,13 +714,13 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>2605679.29</v>
+        <v>1475014.15</v>
       </c>
       <c r="C11">
-        <v>2826007.02</v>
+        <v>1581776.35</v>
       </c>
       <c r="D11">
-        <v>-220327.73</v>
+        <v>-106762.2</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -731,13 +728,13 @@
         <v>14</v>
       </c>
       <c r="B12">
-        <v>958517.72</v>
+        <v>2681722.96</v>
       </c>
       <c r="C12">
-        <v>1039566.86</v>
+        <v>2894310.02</v>
       </c>
       <c r="D12">
-        <v>-81049.14</v>
+        <v>-212587.06</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -745,13 +742,13 @@
         <v>15</v>
       </c>
       <c r="B13">
-        <v>132996.72</v>
+        <v>986490.88</v>
       </c>
       <c r="C13">
-        <v>144077.98</v>
+        <v>1064692.57</v>
       </c>
       <c r="D13">
-        <v>-11081.26</v>
+        <v>-78201.69</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -759,13 +756,13 @@
         <v>16</v>
       </c>
       <c r="B14">
-        <v>556429.55</v>
+        <v>135815.67</v>
       </c>
       <c r="C14">
-        <v>613918.59</v>
+        <v>146413.8</v>
       </c>
       <c r="D14">
-        <v>-57489.04</v>
+        <v>-10598.13</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -773,13 +770,13 @@
         <v>17</v>
       </c>
       <c r="B15">
-        <v>19736.71</v>
+        <v>608988.6800000001</v>
       </c>
       <c r="C15">
-        <v>22044.16</v>
+        <v>671379.25</v>
       </c>
       <c r="D15">
-        <v>-2307.45</v>
+        <v>-62390.57</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -787,13 +784,13 @@
         <v>18</v>
       </c>
       <c r="B16">
-        <v>339053</v>
+        <v>22836.61</v>
       </c>
       <c r="C16">
-        <v>625552.79</v>
+        <v>25315.61</v>
       </c>
       <c r="D16">
-        <v>-286499.79</v>
+        <v>-2479</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -801,13 +798,13 @@
         <v>19</v>
       </c>
       <c r="B17">
-        <v>31674.56</v>
+        <v>286499.79</v>
       </c>
       <c r="C17">
-        <v>60379.87</v>
+        <v>286499.79</v>
       </c>
       <c r="D17">
-        <v>-28705.31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -815,13 +812,13 @@
         <v>20</v>
       </c>
       <c r="B18">
-        <v>1861199.55</v>
+        <v>28705.31</v>
       </c>
       <c r="C18">
-        <v>2018576.52</v>
+        <v>28705.31</v>
       </c>
       <c r="D18">
-        <v>-157376.97</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -829,13 +826,13 @@
         <v>21</v>
       </c>
       <c r="B19">
-        <v>958517.72</v>
+        <v>1915516.5</v>
       </c>
       <c r="C19">
-        <v>1039566.86</v>
+        <v>2067364.4</v>
       </c>
       <c r="D19">
-        <v>-81049.14</v>
+        <v>-151847.9</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -843,13 +840,13 @@
         <v>22</v>
       </c>
       <c r="B20">
-        <v>54000</v>
+        <v>986490.88</v>
       </c>
       <c r="C20">
-        <v>54000</v>
+        <v>1064692.57</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>-78201.69</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -857,13 +854,13 @@
         <v>23</v>
       </c>
       <c r="B21">
-        <v>397566</v>
+        <v>56000</v>
       </c>
       <c r="C21">
-        <v>440926</v>
+        <v>56000</v>
       </c>
       <c r="D21">
-        <v>-43360</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -871,13 +868,13 @@
         <v>24</v>
       </c>
       <c r="B22">
-        <v>8668.219999999999</v>
+        <v>393285.97</v>
       </c>
       <c r="C22">
-        <v>11901.16</v>
+        <v>393285.97</v>
       </c>
       <c r="D22">
-        <v>-3232.94</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -885,13 +882,13 @@
         <v>25</v>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>26396.18</v>
       </c>
       <c r="C23">
-        <v>13960.43</v>
+        <v>26396.18</v>
       </c>
       <c r="D23">
-        <v>-13960.43</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -899,13 +896,13 @@
         <v>26</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>65031.16</v>
       </c>
       <c r="C24">
-        <v>5991.36</v>
+        <v>65031.16</v>
       </c>
       <c r="D24">
-        <v>-5991.36</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -913,13 +910,13 @@
         <v>27</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>27909.22</v>
       </c>
       <c r="C25">
-        <v>436.26</v>
+        <v>27909.22</v>
       </c>
       <c r="D25">
-        <v>-436.26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -927,13 +924,13 @@
         <v>28</v>
       </c>
       <c r="B26">
-        <v>9982915.4</v>
+        <v>2032.22</v>
       </c>
       <c r="C26">
-        <v>10667428.03</v>
+        <v>2032.22</v>
       </c>
       <c r="D26">
-        <v>-684512.63</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -941,13 +938,13 @@
         <v>29</v>
       </c>
       <c r="B27">
-        <v>1083899.59</v>
+        <v>107841.11</v>
       </c>
       <c r="C27">
-        <v>2770346.77</v>
+        <v>107841.11</v>
       </c>
       <c r="D27">
-        <v>-1686447.18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -955,13 +952,13 @@
         <v>30</v>
       </c>
       <c r="B28">
-        <v>0</v>
+        <v>9995310.859999999</v>
       </c>
       <c r="C28">
-        <v>0</v>
+        <v>10805070.07</v>
       </c>
       <c r="D28">
-        <v>0</v>
+        <v>-809759.21</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -969,13 +966,13 @@
         <v>31</v>
       </c>
       <c r="B29">
-        <v>563135.73</v>
+        <v>1601443.78</v>
       </c>
       <c r="C29">
-        <v>2309232.31</v>
+        <v>2468034</v>
       </c>
       <c r="D29">
-        <v>-1746096.58</v>
+        <v>-866590.22</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -983,10 +980,10 @@
         <v>32</v>
       </c>
       <c r="B30">
-        <v>53750</v>
+        <v>312014.11</v>
       </c>
       <c r="C30">
-        <v>53750</v>
+        <v>312014.11</v>
       </c>
       <c r="D30">
         <v>0</v>
@@ -997,13 +994,13 @@
         <v>33</v>
       </c>
       <c r="B31">
-        <v>32482973.87</v>
+        <v>835974.6899999999</v>
       </c>
       <c r="C31">
-        <v>32482973.87</v>
+        <v>2373972.98</v>
       </c>
       <c r="D31">
-        <v>0</v>
+        <v>-1537998.29</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -1011,13 +1008,13 @@
         <v>34</v>
       </c>
       <c r="B32">
-        <v>244538.88</v>
+        <v>4400</v>
       </c>
       <c r="C32">
-        <v>0</v>
+        <v>4400</v>
       </c>
       <c r="D32">
-        <v>244538.88</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -1025,13 +1022,13 @@
         <v>35</v>
       </c>
       <c r="B33">
-        <v>0</v>
+        <v>457508.88</v>
       </c>
       <c r="C33">
-        <v>244538.88</v>
+        <v>239038.88</v>
       </c>
       <c r="D33">
-        <v>-244538.88</v>
+        <v>218470</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -1039,13 +1036,13 @@
         <v>36</v>
       </c>
       <c r="B34">
-        <v>18611994.66</v>
+        <v>239038.88</v>
       </c>
       <c r="C34">
-        <v>18611994.66</v>
+        <v>457508.88</v>
       </c>
       <c r="D34">
-        <v>0</v>
+        <v>-218470</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -1053,10 +1050,10 @@
         <v>37</v>
       </c>
       <c r="B35">
-        <v>1861199.55</v>
+        <v>19155163.82</v>
       </c>
       <c r="C35">
-        <v>1861199.55</v>
+        <v>19155163.82</v>
       </c>
       <c r="D35">
         <v>0</v>
@@ -1067,10 +1064,10 @@
         <v>38</v>
       </c>
       <c r="B36">
-        <v>958517.72</v>
+        <v>1915516.5</v>
       </c>
       <c r="C36">
-        <v>958517.72</v>
+        <v>1915516.5</v>
       </c>
       <c r="D36">
         <v>0</v>
@@ -1081,10 +1078,10 @@
         <v>39</v>
       </c>
       <c r="B37">
-        <v>54000</v>
+        <v>986490.88</v>
       </c>
       <c r="C37">
-        <v>54000</v>
+        <v>986490.88</v>
       </c>
       <c r="D37">
         <v>0</v>
@@ -1095,10 +1092,10 @@
         <v>40</v>
       </c>
       <c r="B38">
-        <v>265566</v>
+        <v>56000</v>
       </c>
       <c r="C38">
-        <v>265566</v>
+        <v>56000</v>
       </c>
       <c r="D38">
         <v>0</v>
@@ -1109,10 +1106,10 @@
         <v>41</v>
       </c>
       <c r="B39">
-        <v>140668.22</v>
+        <v>-0.03</v>
       </c>
       <c r="C39">
-        <v>140668.22</v>
+        <v>-0.03</v>
       </c>
       <c r="D39">
         <v>0</v>
@@ -1123,10 +1120,10 @@
         <v>42</v>
       </c>
       <c r="B40">
-        <v>576166.26</v>
+        <v>202640.67</v>
       </c>
       <c r="C40">
-        <v>576166.26</v>
+        <v>202640.67</v>
       </c>
       <c r="D40">
         <v>0</v>
@@ -1137,10 +1134,10 @@
         <v>43</v>
       </c>
       <c r="B41">
-        <v>370727.56</v>
+        <v>631825.29</v>
       </c>
       <c r="C41">
-        <v>370727.56</v>
+        <v>631825.29</v>
       </c>
       <c r="D41">
         <v>0</v>
@@ -1151,10 +1148,10 @@
         <v>44</v>
       </c>
       <c r="B42">
-        <v>740509.5</v>
+        <v>315205.1</v>
       </c>
       <c r="C42">
-        <v>740509.5</v>
+        <v>315205.1</v>
       </c>
       <c r="D42">
         <v>0</v>
@@ -1165,10 +1162,10 @@
         <v>45</v>
       </c>
       <c r="B43">
-        <v>2677291.14</v>
+        <v>1127007.15</v>
       </c>
       <c r="C43">
-        <v>2677291.14</v>
+        <v>1127007.15</v>
       </c>
       <c r="D43">
         <v>0</v>
@@ -1179,10 +1176,10 @@
         <v>46</v>
       </c>
       <c r="B44">
-        <v>1996554.4</v>
+        <v>4626783.83</v>
       </c>
       <c r="C44">
-        <v>1996554.4</v>
+        <v>4626783.83</v>
       </c>
       <c r="D44">
         <v>0</v>
@@ -1193,10 +1190,10 @@
         <v>47</v>
       </c>
       <c r="B45">
-        <v>87348.53999999999</v>
+        <v>551758.66</v>
       </c>
       <c r="C45">
-        <v>87348.53999999999</v>
+        <v>551758.66</v>
       </c>
       <c r="D45">
         <v>0</v>
@@ -1207,10 +1204,10 @@
         <v>48</v>
       </c>
       <c r="B46">
-        <v>1447894.27</v>
+        <v>76287.66</v>
       </c>
       <c r="C46">
-        <v>1447894.27</v>
+        <v>76287.66</v>
       </c>
       <c r="D46">
         <v>0</v>
@@ -1221,10 +1218,10 @@
         <v>49</v>
       </c>
       <c r="B47">
-        <v>6060.06</v>
+        <v>1379787.82</v>
       </c>
       <c r="C47">
-        <v>6060.06</v>
+        <v>1379787.82</v>
       </c>
       <c r="D47">
         <v>0</v>
@@ -1235,10 +1232,10 @@
         <v>50</v>
       </c>
       <c r="B48">
-        <v>47000</v>
+        <v>6789.6</v>
       </c>
       <c r="C48">
-        <v>47000</v>
+        <v>6789.6</v>
       </c>
       <c r="D48">
         <v>0</v>
@@ -1249,10 +1246,10 @@
         <v>51</v>
       </c>
       <c r="B49">
-        <v>400000</v>
+        <v>28200</v>
       </c>
       <c r="C49">
-        <v>400000</v>
+        <v>28200</v>
       </c>
       <c r="D49">
         <v>0</v>
@@ -1263,10 +1260,10 @@
         <v>52</v>
       </c>
       <c r="B50">
-        <v>499200</v>
+        <v>516000</v>
       </c>
       <c r="C50">
-        <v>499200</v>
+        <v>516000</v>
       </c>
       <c r="D50">
         <v>0</v>
@@ -1277,10 +1274,10 @@
         <v>53</v>
       </c>
       <c r="B51">
-        <v>71366.39999999999</v>
+        <v>169292.62</v>
       </c>
       <c r="C51">
-        <v>71366.39999999999</v>
+        <v>169292.62</v>
       </c>
       <c r="D51">
         <v>0</v>
@@ -1291,10 +1288,10 @@
         <v>54</v>
       </c>
       <c r="B52">
-        <v>374000</v>
+        <v>75752</v>
       </c>
       <c r="C52">
-        <v>374000</v>
+        <v>75752</v>
       </c>
       <c r="D52">
         <v>0</v>
@@ -1305,10 +1302,10 @@
         <v>55</v>
       </c>
       <c r="B53">
-        <v>128190.54</v>
+        <v>20686.52</v>
       </c>
       <c r="C53">
-        <v>128190.54</v>
+        <v>20686.52</v>
       </c>
       <c r="D53">
         <v>0</v>
@@ -1319,10 +1316,10 @@
         <v>56</v>
       </c>
       <c r="B54">
-        <v>24944</v>
+        <v>85080</v>
       </c>
       <c r="C54">
-        <v>24944</v>
+        <v>85080</v>
       </c>
       <c r="D54">
         <v>0</v>
@@ -1333,10 +1330,10 @@
         <v>57</v>
       </c>
       <c r="B55">
-        <v>200000</v>
+        <v>536562</v>
       </c>
       <c r="C55">
-        <v>200000</v>
+        <v>536562</v>
       </c>
       <c r="D55">
         <v>0</v>
@@ -1347,10 +1344,10 @@
         <v>58</v>
       </c>
       <c r="B56">
-        <v>65077.55</v>
+        <v>108700</v>
       </c>
       <c r="C56">
-        <v>65077.55</v>
+        <v>108700</v>
       </c>
       <c r="D56">
         <v>0</v>
@@ -1361,10 +1358,10 @@
         <v>59</v>
       </c>
       <c r="B57">
-        <v>1500</v>
+        <v>193256</v>
       </c>
       <c r="C57">
-        <v>1500</v>
+        <v>193256</v>
       </c>
       <c r="D57">
         <v>0</v>
@@ -1375,10 +1372,10 @@
         <v>60</v>
       </c>
       <c r="B58">
-        <v>594786</v>
+        <v>54028.8</v>
       </c>
       <c r="C58">
-        <v>594786</v>
+        <v>54028.8</v>
       </c>
       <c r="D58">
         <v>0</v>
@@ -1389,10 +1386,10 @@
         <v>61</v>
       </c>
       <c r="B59">
-        <v>47300</v>
+        <v>125400</v>
       </c>
       <c r="C59">
-        <v>47300</v>
+        <v>125400</v>
       </c>
       <c r="D59">
         <v>0</v>
@@ -1403,10 +1400,10 @@
         <v>62</v>
       </c>
       <c r="B60">
-        <v>113488.8</v>
+        <v>107841.11</v>
       </c>
       <c r="C60">
-        <v>113488.8</v>
+        <v>107841.11</v>
       </c>
       <c r="D60">
         <v>0</v>
@@ -1417,10 +1414,10 @@
         <v>63</v>
       </c>
       <c r="B61">
-        <v>41947.2</v>
+        <v>313938.2</v>
       </c>
       <c r="C61">
-        <v>41947.2</v>
+        <v>313938.2</v>
       </c>
       <c r="D61">
         <v>0</v>
@@ -1431,26 +1428,12 @@
         <v>64</v>
       </c>
       <c r="B62">
-        <v>79404</v>
+        <v>33365994.2</v>
       </c>
       <c r="C62">
-        <v>79404</v>
+        <v>33365994.2</v>
       </c>
       <c r="D62">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4">
-      <c r="A63" t="s">
-        <v>65</v>
-      </c>
-      <c r="B63">
-        <v>32482702.37</v>
-      </c>
-      <c r="C63">
-        <v>32482702.37</v>
-      </c>
-      <c r="D63">
         <v>0</v>
       </c>
     </row>

</xml_diff>